<commit_message>
Refactor competitive baselines and update metrics
</commit_message>
<xml_diff>
--- a/Combined Metrics/competitive_baselines.xlsx
+++ b/Combined Metrics/competitive_baselines.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="AE_vs_FixedDefault" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="AE_vs_NearestNeighbor" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="SingleCriterionArgmax" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="BestSingleCriterion" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="PairedTests_AE_vs_baselines" sheetId="4" state="visible" r:id="rId4"/>
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T17"/>
+  <dimension ref="A1:N17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -462,60 +462,30 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>FD_tau</t>
+          <t>NN_tau</t>
         </is>
       </c>
       <c r="J1" t="inlineStr">
         <is>
-          <t>FD_top1</t>
+          <t>NN_top1</t>
         </is>
       </c>
       <c r="K1" t="inlineStr">
         <is>
-          <t>NN_tau</t>
+          <t>d_tau_NN</t>
         </is>
       </c>
       <c r="L1" t="inlineStr">
         <is>
-          <t>NN_top1</t>
+          <t>d_top1_NN</t>
         </is>
       </c>
       <c r="M1" t="inlineStr">
         <is>
-          <t>d_tau</t>
+          <t>AE_beats_NN_tau</t>
         </is>
       </c>
       <c r="N1" t="inlineStr">
-        <is>
-          <t>d_top1</t>
-        </is>
-      </c>
-      <c r="O1" t="inlineStr">
-        <is>
-          <t>AE_beats_FD_tau</t>
-        </is>
-      </c>
-      <c r="P1" t="inlineStr">
-        <is>
-          <t>AE_beats_FD_top1</t>
-        </is>
-      </c>
-      <c r="Q1" t="inlineStr">
-        <is>
-          <t>d_tau_NN</t>
-        </is>
-      </c>
-      <c r="R1" t="inlineStr">
-        <is>
-          <t>d_top1_NN</t>
-        </is>
-      </c>
-      <c r="S1" t="inlineStr">
-        <is>
-          <t>AE_beats_NN_tau</t>
-        </is>
-      </c>
-      <c r="T1" t="inlineStr">
         <is>
           <t>AE_beats_NN_top1</t>
         </is>
@@ -551,39 +521,21 @@
         <v>194.8</v>
       </c>
       <c r="I2" t="n">
-        <v>0.5795</v>
+        <v>0.3744</v>
       </c>
       <c r="J2" t="n">
-        <v>0.6359</v>
+        <v>0.6462</v>
       </c>
       <c r="K2" t="n">
-        <v>0.3744</v>
+        <v>-0.1214</v>
       </c>
       <c r="L2" t="n">
-        <v>0.6462</v>
-      </c>
-      <c r="M2" t="n">
-        <v>-0.3265</v>
-      </c>
-      <c r="N2" t="n">
-        <v>-0.15282</v>
-      </c>
-      <c r="O2" t="b">
-        <v>0</v>
-      </c>
-      <c r="P2" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q2" t="n">
-        <v>-0.1214</v>
-      </c>
-      <c r="R2" t="n">
         <v>-0.16312</v>
       </c>
-      <c r="S2" t="b">
-        <v>0</v>
-      </c>
-      <c r="T2" t="b">
+      <c r="M2" t="b">
+        <v>0</v>
+      </c>
+      <c r="N2" t="b">
         <v>0</v>
       </c>
     </row>
@@ -617,39 +569,21 @@
         <v>70</v>
       </c>
       <c r="I3" t="n">
-        <v>0.7905</v>
+        <v>0.181</v>
       </c>
       <c r="J3" t="n">
-        <v>0.7714</v>
+        <v>0.5143</v>
       </c>
       <c r="K3" t="n">
-        <v>0.181</v>
+        <v>-0.15054</v>
       </c>
       <c r="L3" t="n">
-        <v>0.5143</v>
-      </c>
-      <c r="M3" t="n">
-        <v>-0.7600399999999999</v>
-      </c>
-      <c r="N3" t="n">
-        <v>-0.4742399999999999</v>
-      </c>
-      <c r="O3" t="b">
-        <v>0</v>
-      </c>
-      <c r="P3" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q3" t="n">
-        <v>-0.15054</v>
-      </c>
-      <c r="R3" t="n">
         <v>-0.2171399999999999</v>
       </c>
-      <c r="S3" t="b">
-        <v>0</v>
-      </c>
-      <c r="T3" t="b">
+      <c r="M3" t="b">
+        <v>0</v>
+      </c>
+      <c r="N3" t="b">
         <v>0</v>
       </c>
     </row>
@@ -683,39 +617,21 @@
         <v>64.8</v>
       </c>
       <c r="I4" t="n">
-        <v>0.1795</v>
+        <v>0.4667</v>
       </c>
       <c r="J4" t="n">
-        <v>0.3231</v>
+        <v>0.7231</v>
       </c>
       <c r="K4" t="n">
-        <v>0.4667</v>
+        <v>-0.1795</v>
       </c>
       <c r="L4" t="n">
-        <v>0.7231</v>
-      </c>
-      <c r="M4" t="n">
-        <v>0.1077</v>
-      </c>
-      <c r="N4" t="n">
-        <v>0.2769</v>
-      </c>
-      <c r="O4" t="b">
-        <v>1</v>
-      </c>
-      <c r="P4" t="b">
-        <v>1</v>
-      </c>
-      <c r="Q4" t="n">
-        <v>-0.1795</v>
-      </c>
-      <c r="R4" t="n">
         <v>-0.1231</v>
       </c>
-      <c r="S4" t="b">
-        <v>0</v>
-      </c>
-      <c r="T4" t="b">
+      <c r="M4" t="b">
+        <v>0</v>
+      </c>
+      <c r="N4" t="b">
         <v>0</v>
       </c>
     </row>
@@ -749,39 +665,21 @@
         <v>60</v>
       </c>
       <c r="I5" t="n">
-        <v>0.7667</v>
+        <v>0.5</v>
       </c>
       <c r="J5" t="n">
-        <v>0.8167</v>
+        <v>0.7167</v>
       </c>
       <c r="K5" t="n">
-        <v>0.5</v>
+        <v>-0.02444000000000007</v>
       </c>
       <c r="L5" t="n">
-        <v>0.7167</v>
-      </c>
-      <c r="M5" t="n">
-        <v>-0.2911400000000001</v>
-      </c>
-      <c r="N5" t="n">
-        <v>-0.2433399999999999</v>
-      </c>
-      <c r="O5" t="b">
-        <v>0</v>
-      </c>
-      <c r="P5" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q5" t="n">
-        <v>-0.02444000000000007</v>
-      </c>
-      <c r="R5" t="n">
         <v>-0.1433399999999999</v>
       </c>
-      <c r="S5" t="b">
-        <v>0</v>
-      </c>
-      <c r="T5" t="b">
+      <c r="M5" t="b">
+        <v>0</v>
+      </c>
+      <c r="N5" t="b">
         <v>0</v>
       </c>
     </row>
@@ -815,39 +713,21 @@
         <v>195</v>
       </c>
       <c r="I6" t="n">
-        <v>0.5795</v>
+        <v>0.3744</v>
       </c>
       <c r="J6" t="n">
-        <v>0.6359</v>
+        <v>0.6462</v>
       </c>
       <c r="K6" t="n">
-        <v>0.3744</v>
+        <v>-0.07594000000000001</v>
       </c>
       <c r="L6" t="n">
-        <v>0.6462</v>
-      </c>
-      <c r="M6" t="n">
-        <v>-0.28104</v>
-      </c>
-      <c r="N6" t="n">
-        <v>-0.1610400000000001</v>
-      </c>
-      <c r="O6" t="b">
-        <v>0</v>
-      </c>
-      <c r="P6" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q6" t="n">
-        <v>-0.07594000000000001</v>
-      </c>
-      <c r="R6" t="n">
         <v>-0.17134</v>
       </c>
-      <c r="S6" t="b">
-        <v>0</v>
-      </c>
-      <c r="T6" t="b">
+      <c r="M6" t="b">
+        <v>0</v>
+      </c>
+      <c r="N6" t="b">
         <v>0</v>
       </c>
     </row>
@@ -881,39 +761,21 @@
         <v>70</v>
       </c>
       <c r="I7" t="n">
-        <v>0.7905</v>
+        <v>0.181</v>
       </c>
       <c r="J7" t="n">
-        <v>0.7714</v>
+        <v>0.5143</v>
       </c>
       <c r="K7" t="n">
-        <v>0.181</v>
+        <v>-0.2991</v>
       </c>
       <c r="L7" t="n">
-        <v>0.5143</v>
-      </c>
-      <c r="M7" t="n">
-        <v>-0.9086</v>
-      </c>
-      <c r="N7" t="n">
-        <v>-0.61998</v>
-      </c>
-      <c r="O7" t="b">
-        <v>0</v>
-      </c>
-      <c r="P7" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q7" t="n">
-        <v>-0.2991</v>
-      </c>
-      <c r="R7" t="n">
         <v>-0.36288</v>
       </c>
-      <c r="S7" t="b">
-        <v>0</v>
-      </c>
-      <c r="T7" t="b">
+      <c r="M7" t="b">
+        <v>0</v>
+      </c>
+      <c r="N7" t="b">
         <v>0</v>
       </c>
     </row>
@@ -947,39 +809,21 @@
         <v>65</v>
       </c>
       <c r="I8" t="n">
-        <v>0.1795</v>
+        <v>0.4667</v>
       </c>
       <c r="J8" t="n">
-        <v>0.3231</v>
+        <v>0.7231</v>
       </c>
       <c r="K8" t="n">
-        <v>0.4667</v>
+        <v>-0.16412</v>
       </c>
       <c r="L8" t="n">
-        <v>0.7231</v>
-      </c>
-      <c r="M8" t="n">
-        <v>0.12308</v>
-      </c>
-      <c r="N8" t="n">
-        <v>0.2215</v>
-      </c>
-      <c r="O8" t="b">
-        <v>1</v>
-      </c>
-      <c r="P8" t="b">
-        <v>1</v>
-      </c>
-      <c r="Q8" t="n">
-        <v>-0.16412</v>
-      </c>
-      <c r="R8" t="n">
         <v>-0.1785</v>
       </c>
-      <c r="S8" t="b">
-        <v>0</v>
-      </c>
-      <c r="T8" t="b">
+      <c r="M8" t="b">
+        <v>0</v>
+      </c>
+      <c r="N8" t="b">
         <v>0</v>
       </c>
     </row>
@@ -1013,39 +857,21 @@
         <v>60</v>
       </c>
       <c r="I9" t="n">
-        <v>0.7667</v>
+        <v>0.5</v>
       </c>
       <c r="J9" t="n">
-        <v>0.8167</v>
+        <v>0.7167</v>
       </c>
       <c r="K9" t="n">
-        <v>0.5</v>
+        <v>0.28002</v>
       </c>
       <c r="L9" t="n">
-        <v>0.7167</v>
-      </c>
-      <c r="M9" t="n">
-        <v>0.01332</v>
-      </c>
-      <c r="N9" t="n">
-        <v>-0.04001999999999994</v>
-      </c>
-      <c r="O9" t="b">
+        <v>0.05998000000000003</v>
+      </c>
+      <c r="M9" t="b">
         <v>1</v>
       </c>
-      <c r="P9" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q9" t="n">
-        <v>0.28002</v>
-      </c>
-      <c r="R9" t="n">
-        <v>0.05998000000000003</v>
-      </c>
-      <c r="S9" t="b">
-        <v>1</v>
-      </c>
-      <c r="T9" t="b">
+      <c r="N9" t="b">
         <v>1</v>
       </c>
     </row>
@@ -1079,39 +905,21 @@
         <v>195</v>
       </c>
       <c r="I10" t="n">
-        <v>0.5795</v>
+        <v>0.3744</v>
       </c>
       <c r="J10" t="n">
-        <v>0.6359</v>
+        <v>0.6462</v>
       </c>
       <c r="K10" t="n">
-        <v>0.3744</v>
+        <v>-0.14022</v>
       </c>
       <c r="L10" t="n">
-        <v>0.6462</v>
-      </c>
-      <c r="M10" t="n">
-        <v>-0.34532</v>
-      </c>
-      <c r="N10" t="n">
-        <v>-0.17128</v>
-      </c>
-      <c r="O10" t="b">
-        <v>0</v>
-      </c>
-      <c r="P10" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q10" t="n">
-        <v>-0.14022</v>
-      </c>
-      <c r="R10" t="n">
         <v>-0.18158</v>
       </c>
-      <c r="S10" t="b">
-        <v>0</v>
-      </c>
-      <c r="T10" t="b">
+      <c r="M10" t="b">
+        <v>0</v>
+      </c>
+      <c r="N10" t="b">
         <v>0</v>
       </c>
     </row>
@@ -1145,39 +953,21 @@
         <v>70</v>
       </c>
       <c r="I11" t="n">
-        <v>0.7905</v>
+        <v>0.181</v>
       </c>
       <c r="J11" t="n">
-        <v>0.7714</v>
+        <v>0.5143</v>
       </c>
       <c r="K11" t="n">
-        <v>0.181</v>
+        <v>0.02090000000000003</v>
       </c>
       <c r="L11" t="n">
-        <v>0.5143</v>
-      </c>
-      <c r="M11" t="n">
-        <v>-0.5886</v>
-      </c>
-      <c r="N11" t="n">
-        <v>-0.36852</v>
-      </c>
-      <c r="O11" t="b">
-        <v>0</v>
-      </c>
-      <c r="P11" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q11" t="n">
-        <v>0.02090000000000003</v>
-      </c>
-      <c r="R11" t="n">
         <v>-0.11142</v>
       </c>
-      <c r="S11" t="b">
+      <c r="M11" t="b">
         <v>1</v>
       </c>
-      <c r="T11" t="b">
+      <c r="N11" t="b">
         <v>0</v>
       </c>
     </row>
@@ -1211,39 +1001,21 @@
         <v>65</v>
       </c>
       <c r="I12" t="n">
-        <v>0.1795</v>
+        <v>0.4667</v>
       </c>
       <c r="J12" t="n">
-        <v>0.3231</v>
+        <v>0.7231</v>
       </c>
       <c r="K12" t="n">
-        <v>0.4667</v>
+        <v>-0.5395</v>
       </c>
       <c r="L12" t="n">
-        <v>0.7231</v>
-      </c>
-      <c r="M12" t="n">
-        <v>-0.2523</v>
-      </c>
-      <c r="N12" t="n">
-        <v>0.003059999999999952</v>
-      </c>
-      <c r="O12" t="b">
-        <v>0</v>
-      </c>
-      <c r="P12" t="b">
-        <v>1</v>
-      </c>
-      <c r="Q12" t="n">
-        <v>-0.5395</v>
-      </c>
-      <c r="R12" t="n">
         <v>-0.39694</v>
       </c>
-      <c r="S12" t="b">
-        <v>0</v>
-      </c>
-      <c r="T12" t="b">
+      <c r="M12" t="b">
+        <v>0</v>
+      </c>
+      <c r="N12" t="b">
         <v>0</v>
       </c>
     </row>
@@ -1277,39 +1049,21 @@
         <v>60</v>
       </c>
       <c r="I13" t="n">
-        <v>0.7667</v>
+        <v>0.5</v>
       </c>
       <c r="J13" t="n">
-        <v>0.8167</v>
+        <v>0.7167</v>
       </c>
       <c r="K13" t="n">
-        <v>0.5</v>
+        <v>0.10442</v>
       </c>
       <c r="L13" t="n">
-        <v>0.7167</v>
-      </c>
-      <c r="M13" t="n">
-        <v>-0.1622800000000001</v>
-      </c>
-      <c r="N13" t="n">
-        <v>-0.13002</v>
-      </c>
-      <c r="O13" t="b">
-        <v>0</v>
-      </c>
-      <c r="P13" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q13" t="n">
-        <v>0.10442</v>
-      </c>
-      <c r="R13" t="n">
         <v>-0.03002000000000005</v>
       </c>
-      <c r="S13" t="b">
+      <c r="M13" t="b">
         <v>1</v>
       </c>
-      <c r="T13" t="b">
+      <c r="N13" t="b">
         <v>0</v>
       </c>
     </row>
@@ -1343,39 +1097,21 @@
         <v>195</v>
       </c>
       <c r="I14" t="n">
-        <v>0.5795</v>
+        <v>0.3744</v>
       </c>
       <c r="J14" t="n">
-        <v>0.6359</v>
+        <v>0.6462</v>
       </c>
       <c r="K14" t="n">
-        <v>0.3744</v>
+        <v>-0.22704</v>
       </c>
       <c r="L14" t="n">
-        <v>0.6462</v>
-      </c>
-      <c r="M14" t="n">
-        <v>-0.43214</v>
-      </c>
-      <c r="N14" t="n">
-        <v>-0.19692</v>
-      </c>
-      <c r="O14" t="b">
-        <v>0</v>
-      </c>
-      <c r="P14" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q14" t="n">
-        <v>-0.22704</v>
-      </c>
-      <c r="R14" t="n">
         <v>-0.20722</v>
       </c>
-      <c r="S14" t="b">
-        <v>0</v>
-      </c>
-      <c r="T14" t="b">
+      <c r="M14" t="b">
+        <v>0</v>
+      </c>
+      <c r="N14" t="b">
         <v>0</v>
       </c>
     </row>
@@ -1409,39 +1145,21 @@
         <v>70</v>
       </c>
       <c r="I15" t="n">
-        <v>0.7905</v>
+        <v>0.181</v>
       </c>
       <c r="J15" t="n">
-        <v>0.7714</v>
+        <v>0.5143</v>
       </c>
       <c r="K15" t="n">
-        <v>0.181</v>
+        <v>-0.12196</v>
       </c>
       <c r="L15" t="n">
-        <v>0.5143</v>
-      </c>
-      <c r="M15" t="n">
-        <v>-0.73146</v>
-      </c>
-      <c r="N15" t="n">
-        <v>-0.41712</v>
-      </c>
-      <c r="O15" t="b">
-        <v>0</v>
-      </c>
-      <c r="P15" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q15" t="n">
-        <v>-0.12196</v>
-      </c>
-      <c r="R15" t="n">
         <v>-0.16002</v>
       </c>
-      <c r="S15" t="b">
-        <v>0</v>
-      </c>
-      <c r="T15" t="b">
+      <c r="M15" t="b">
+        <v>0</v>
+      </c>
+      <c r="N15" t="b">
         <v>0</v>
       </c>
     </row>
@@ -1475,39 +1193,21 @@
         <v>65</v>
       </c>
       <c r="I16" t="n">
-        <v>0.1795</v>
+        <v>0.4667</v>
       </c>
       <c r="J16" t="n">
-        <v>0.3231</v>
+        <v>0.7231</v>
       </c>
       <c r="K16" t="n">
-        <v>0.4667</v>
+        <v>-0.31798</v>
       </c>
       <c r="L16" t="n">
-        <v>0.7231</v>
-      </c>
-      <c r="M16" t="n">
-        <v>-0.03077999999999997</v>
-      </c>
-      <c r="N16" t="n">
-        <v>0.15074</v>
-      </c>
-      <c r="O16" t="b">
-        <v>0</v>
-      </c>
-      <c r="P16" t="b">
-        <v>1</v>
-      </c>
-      <c r="Q16" t="n">
-        <v>-0.31798</v>
-      </c>
-      <c r="R16" t="n">
         <v>-0.2492599999999999</v>
       </c>
-      <c r="S16" t="b">
-        <v>0</v>
-      </c>
-      <c r="T16" t="b">
+      <c r="M16" t="b">
+        <v>0</v>
+      </c>
+      <c r="N16" t="b">
         <v>0</v>
       </c>
     </row>
@@ -1541,39 +1241,21 @@
         <v>60</v>
       </c>
       <c r="I17" t="n">
-        <v>0.7667</v>
+        <v>0.5</v>
       </c>
       <c r="J17" t="n">
-        <v>0.8167</v>
+        <v>0.7167</v>
       </c>
       <c r="K17" t="n">
-        <v>0.5</v>
+        <v>-0.2511</v>
       </c>
       <c r="L17" t="n">
-        <v>0.7167</v>
-      </c>
-      <c r="M17" t="n">
-        <v>-0.5178</v>
-      </c>
-      <c r="N17" t="n">
-        <v>-0.3167</v>
-      </c>
-      <c r="O17" t="b">
-        <v>0</v>
-      </c>
-      <c r="P17" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q17" t="n">
-        <v>-0.2511</v>
-      </c>
-      <c r="R17" t="n">
         <v>-0.2167</v>
       </c>
-      <c r="S17" t="b">
-        <v>0</v>
-      </c>
-      <c r="T17" t="b">
+      <c r="M17" t="b">
+        <v>0</v>
+      </c>
+      <c r="N17" t="b">
         <v>0</v>
       </c>
     </row>
@@ -1985,7 +1667,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O17"/>
+  <dimension ref="A1:O9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2073,7 +1755,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>FixedDefault</t>
+          <t>NearestNeighbor</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -2088,34 +1770,34 @@
         <v>195</v>
       </c>
       <c r="F2" t="n">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="G2" t="n">
         <v>0.2341880341880342</v>
       </c>
       <c r="H2" t="n">
-        <v>0.5794871794871795</v>
+        <v>0.3743589743589744</v>
       </c>
       <c r="I2" t="n">
-        <v>-0.3452991452991453</v>
+        <v>-0.1401709401709402</v>
       </c>
       <c r="J2" t="n">
-        <v>3316</v>
+        <v>5977</v>
       </c>
       <c r="K2" t="n">
-        <v>1.039430597158424e-10</v>
+        <v>0.02529356595850657</v>
       </c>
       <c r="L2" t="n">
-        <v>-0.56440065681445</v>
+        <v>-0.1965317919075145</v>
       </c>
       <c r="M2" t="n">
-        <v>1.559145895737636e-09</v>
+        <v>0.05058713191701314</v>
       </c>
       <c r="N2" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O2" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
     </row>
     <row r="3">
@@ -2126,7 +1808,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>FixedDefault</t>
+          <t>NearestNeighbor</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -2141,40 +1823,40 @@
         <v>195</v>
       </c>
       <c r="F3" t="n">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="G3" t="n">
         <v>0.4646153846153846</v>
       </c>
       <c r="H3" t="n">
-        <v>0.6358974358974359</v>
+        <v>0.6461538461538462</v>
       </c>
       <c r="I3" t="n">
-        <v>-0.1712820512820513</v>
+        <v>-0.1815384615384615</v>
       </c>
       <c r="J3" t="n">
-        <v>3350.5</v>
+        <v>3327</v>
       </c>
       <c r="K3" t="n">
-        <v>0.000178522394952922</v>
+        <v>4.004240568013924e-05</v>
       </c>
       <c r="L3" t="n">
-        <v>-0.3581417624521073</v>
+        <v>-0.3883066740209598</v>
       </c>
       <c r="M3" t="n">
-        <v>0.001249656764670454</v>
+        <v>0.0002002120284006962</v>
       </c>
       <c r="N3" t="b">
         <v>1</v>
       </c>
       <c r="O3" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>gptoss</t>
+          <t>qwen</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -2194,40 +1876,40 @@
         <v>195</v>
       </c>
       <c r="F4" t="n">
-        <v>172</v>
+        <v>183</v>
       </c>
       <c r="G4" t="n">
-        <v>0.2341880341880342</v>
+        <v>0.1473504273504273</v>
       </c>
       <c r="H4" t="n">
         <v>0.3743589743589744</v>
       </c>
       <c r="I4" t="n">
-        <v>-0.1401709401709402</v>
+        <v>-0.227008547008547</v>
       </c>
       <c r="J4" t="n">
-        <v>5977</v>
+        <v>5330</v>
       </c>
       <c r="K4" t="n">
-        <v>0.02529356595850657</v>
+        <v>1.66098943316757e-05</v>
       </c>
       <c r="L4" t="n">
-        <v>-0.1965317919075145</v>
+        <v>-0.3668329769541459</v>
       </c>
       <c r="M4" t="n">
-        <v>0.05058713191701314</v>
+        <v>0.0001162692603217299</v>
       </c>
       <c r="N4" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O4" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>gptoss</t>
+          <t>qwen</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -2247,45 +1929,45 @@
         <v>195</v>
       </c>
       <c r="F5" t="n">
-        <v>147</v>
+        <v>160</v>
       </c>
       <c r="G5" t="n">
-        <v>0.4646153846153846</v>
+        <v>0.4389743589743589</v>
       </c>
       <c r="H5" t="n">
         <v>0.6461538461538462</v>
       </c>
       <c r="I5" t="n">
-        <v>-0.1815384615384615</v>
+        <v>-0.2071794871794872</v>
       </c>
       <c r="J5" t="n">
-        <v>3327</v>
+        <v>3652</v>
       </c>
       <c r="K5" t="n">
-        <v>4.004240568013924e-05</v>
+        <v>1.870478723369979e-06</v>
       </c>
       <c r="L5" t="n">
-        <v>-0.3883066740209598</v>
+        <v>-0.4329192546583851</v>
       </c>
       <c r="M5" t="n">
-        <v>0.0003203392454411139</v>
+        <v>1.496382978695983e-05</v>
       </c>
       <c r="N5" t="b">
         <v>1</v>
       </c>
       <c r="O5" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>qwen</t>
+          <t>deepseek</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>FixedDefault</t>
+          <t>NearestNeighbor</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -2300,45 +1982,45 @@
         <v>195</v>
       </c>
       <c r="F6" t="n">
-        <v>185</v>
+        <v>166</v>
       </c>
       <c r="G6" t="n">
-        <v>0.1473504273504273</v>
+        <v>0.252991452991453</v>
       </c>
       <c r="H6" t="n">
-        <v>0.5794871794871795</v>
+        <v>0.3743589743589744</v>
       </c>
       <c r="I6" t="n">
-        <v>-0.4321367521367522</v>
+        <v>-0.1213675213675214</v>
       </c>
       <c r="J6" t="n">
-        <v>3454</v>
+        <v>5262</v>
       </c>
       <c r="K6" t="n">
-        <v>1.602005184919525e-12</v>
+        <v>0.007094014698653285</v>
       </c>
       <c r="L6" t="n">
-        <v>-0.5984888113920372</v>
+        <v>-0.2407474208210086</v>
       </c>
       <c r="M6" t="n">
-        <v>2.563208295871241e-11</v>
+        <v>0.02128204409595986</v>
       </c>
       <c r="N6" t="b">
         <v>1</v>
       </c>
       <c r="O6" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>qwen</t>
+          <t>deepseek</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>FixedDefault</t>
+          <t>NearestNeighbor</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -2353,40 +2035,40 @@
         <v>195</v>
       </c>
       <c r="F7" t="n">
-        <v>167</v>
+        <v>137</v>
       </c>
       <c r="G7" t="n">
-        <v>0.4389743589743589</v>
+        <v>0.4830769230769231</v>
       </c>
       <c r="H7" t="n">
-        <v>0.6358974358974359</v>
+        <v>0.6461538461538462</v>
       </c>
       <c r="I7" t="n">
-        <v>-0.196923076923077</v>
+        <v>-0.1630769230769231</v>
       </c>
       <c r="J7" t="n">
-        <v>4438</v>
+        <v>2782.5</v>
       </c>
       <c r="K7" t="n">
-        <v>3.548621274296505e-05</v>
+        <v>2.729570298871321e-05</v>
       </c>
       <c r="L7" t="n">
-        <v>-0.3672654690618762</v>
+        <v>-0.4112980006347192</v>
       </c>
       <c r="M7" t="n">
-        <v>0.0003193759146866854</v>
+        <v>0.0001637742179322793</v>
       </c>
       <c r="N7" t="b">
         <v>1</v>
       </c>
       <c r="O7" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>qwen</t>
+          <t>gemini</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -2406,40 +2088,40 @@
         <v>195</v>
       </c>
       <c r="F8" t="n">
-        <v>183</v>
+        <v>132</v>
       </c>
       <c r="G8" t="n">
-        <v>0.1473504273504273</v>
+        <v>0.2984615384615385</v>
       </c>
       <c r="H8" t="n">
         <v>0.3743589743589744</v>
       </c>
       <c r="I8" t="n">
-        <v>-0.227008547008547</v>
+        <v>-0.0758974358974359</v>
       </c>
       <c r="J8" t="n">
-        <v>5330</v>
+        <v>3845.5</v>
       </c>
       <c r="K8" t="n">
-        <v>1.66098943316757e-05</v>
+        <v>0.2158723041617826</v>
       </c>
       <c r="L8" t="n">
-        <v>-0.3668329769541459</v>
+        <v>-0.1238323080428344</v>
       </c>
       <c r="M8" t="n">
-        <v>0.0001993187319801084</v>
+        <v>0.2158723041617826</v>
       </c>
       <c r="N8" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O8" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>qwen</t>
+          <t>gemini</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -2459,458 +2141,34 @@
         <v>195</v>
       </c>
       <c r="F9" t="n">
-        <v>160</v>
+        <v>96</v>
       </c>
       <c r="G9" t="n">
-        <v>0.4389743589743589</v>
+        <v>0.4748717948717948</v>
       </c>
       <c r="H9" t="n">
         <v>0.6461538461538462</v>
       </c>
       <c r="I9" t="n">
-        <v>-0.2071794871794872</v>
+        <v>-0.1712820512820513</v>
       </c>
       <c r="J9" t="n">
-        <v>3652</v>
+        <v>1367.5</v>
       </c>
       <c r="K9" t="n">
-        <v>1.870478723369979e-06</v>
+        <v>0.0002519173754712348</v>
       </c>
       <c r="L9" t="n">
-        <v>-0.4329192546583851</v>
+        <v>-0.4125859106529209</v>
       </c>
       <c r="M9" t="n">
-        <v>2.431622340380973e-05</v>
+        <v>0.001007669501884939</v>
       </c>
       <c r="N9" t="b">
         <v>1</v>
       </c>
       <c r="O9" t="n">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>deepseek</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>FixedDefault</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>tau</t>
-        </is>
-      </c>
-      <c r="D10" t="n">
-        <v>5</v>
-      </c>
-      <c r="E10" t="n">
-        <v>195</v>
-      </c>
-      <c r="F10" t="n">
-        <v>178</v>
-      </c>
-      <c r="G10" t="n">
-        <v>0.252991452991453</v>
-      </c>
-      <c r="H10" t="n">
-        <v>0.5794871794871795</v>
-      </c>
-      <c r="I10" t="n">
-        <v>-0.3264957264957265</v>
-      </c>
-      <c r="J10" t="n">
-        <v>3865.5</v>
-      </c>
-      <c r="K10" t="n">
-        <v>2.53773582272301e-09</v>
-      </c>
-      <c r="L10" t="n">
-        <v>-0.5147197288305819</v>
-      </c>
-      <c r="M10" t="n">
-        <v>3.552830151812214e-08</v>
-      </c>
-      <c r="N10" t="b">
-        <v>1</v>
-      </c>
-      <c r="O10" t="n">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>deepseek</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>FixedDefault</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>Top-1</t>
-        </is>
-      </c>
-      <c r="D11" t="n">
-        <v>5</v>
-      </c>
-      <c r="E11" t="n">
-        <v>195</v>
-      </c>
-      <c r="F11" t="n">
-        <v>164</v>
-      </c>
-      <c r="G11" t="n">
-        <v>0.4830769230769231</v>
-      </c>
-      <c r="H11" t="n">
-        <v>0.6358974358974359</v>
-      </c>
-      <c r="I11" t="n">
-        <v>-0.1528205128205128</v>
-      </c>
-      <c r="J11" t="n">
-        <v>4983.5</v>
-      </c>
-      <c r="K11" t="n">
-        <v>0.003275419188556191</v>
-      </c>
-      <c r="L11" t="n">
-        <v>-0.2633407243163341</v>
-      </c>
-      <c r="M11" t="n">
-        <v>0.01310167675422476</v>
-      </c>
-      <c r="N11" t="b">
-        <v>1</v>
-      </c>
-      <c r="O11" t="n">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>deepseek</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>NearestNeighbor</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>tau</t>
-        </is>
-      </c>
-      <c r="D12" t="n">
-        <v>5</v>
-      </c>
-      <c r="E12" t="n">
-        <v>195</v>
-      </c>
-      <c r="F12" t="n">
-        <v>166</v>
-      </c>
-      <c r="G12" t="n">
-        <v>0.252991452991453</v>
-      </c>
-      <c r="H12" t="n">
-        <v>0.3743589743589744</v>
-      </c>
-      <c r="I12" t="n">
-        <v>-0.1213675213675214</v>
-      </c>
-      <c r="J12" t="n">
-        <v>5262</v>
-      </c>
-      <c r="K12" t="n">
-        <v>0.007094014698653285</v>
-      </c>
-      <c r="L12" t="n">
-        <v>-0.2407474208210086</v>
-      </c>
-      <c r="M12" t="n">
-        <v>0.02128204409595986</v>
-      </c>
-      <c r="N12" t="b">
-        <v>1</v>
-      </c>
-      <c r="O12" t="n">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>deepseek</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>NearestNeighbor</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>Top-1</t>
-        </is>
-      </c>
-      <c r="D13" t="n">
-        <v>5</v>
-      </c>
-      <c r="E13" t="n">
-        <v>195</v>
-      </c>
-      <c r="F13" t="n">
-        <v>137</v>
-      </c>
-      <c r="G13" t="n">
-        <v>0.4830769230769231</v>
-      </c>
-      <c r="H13" t="n">
-        <v>0.6461538461538462</v>
-      </c>
-      <c r="I13" t="n">
-        <v>-0.1630769230769231</v>
-      </c>
-      <c r="J13" t="n">
-        <v>2782.5</v>
-      </c>
-      <c r="K13" t="n">
-        <v>2.729570298871321e-05</v>
-      </c>
-      <c r="L13" t="n">
-        <v>-0.4112980006347192</v>
-      </c>
-      <c r="M13" t="n">
-        <v>0.0002729570298871322</v>
-      </c>
-      <c r="N13" t="b">
-        <v>1</v>
-      </c>
-      <c r="O13" t="n">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>gemini</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>FixedDefault</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>tau</t>
-        </is>
-      </c>
-      <c r="D14" t="n">
-        <v>5</v>
-      </c>
-      <c r="E14" t="n">
-        <v>195</v>
-      </c>
-      <c r="F14" t="n">
-        <v>137</v>
-      </c>
-      <c r="G14" t="n">
-        <v>0.2984615384615385</v>
-      </c>
-      <c r="H14" t="n">
-        <v>0.5794871794871795</v>
-      </c>
-      <c r="I14" t="n">
-        <v>-0.281025641025641</v>
-      </c>
-      <c r="J14" t="n">
-        <v>2748.5</v>
-      </c>
-      <c r="K14" t="n">
-        <v>2.009013227721001e-05</v>
-      </c>
-      <c r="L14" t="n">
-        <v>-0.4184914841849148</v>
-      </c>
-      <c r="M14" t="n">
-        <v>0.0002209914550493101</v>
-      </c>
-      <c r="N14" t="b">
-        <v>1</v>
-      </c>
-      <c r="O14" t="n">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>gemini</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>FixedDefault</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>Top-1</t>
-        </is>
-      </c>
-      <c r="D15" t="n">
-        <v>5</v>
-      </c>
-      <c r="E15" t="n">
-        <v>195</v>
-      </c>
-      <c r="F15" t="n">
-        <v>114</v>
-      </c>
-      <c r="G15" t="n">
-        <v>0.4748717948717948</v>
-      </c>
-      <c r="H15" t="n">
-        <v>0.6358974358974359</v>
-      </c>
-      <c r="I15" t="n">
-        <v>-0.161025641025641</v>
-      </c>
-      <c r="J15" t="n">
-        <v>2220</v>
-      </c>
-      <c r="K15" t="n">
-        <v>0.001632434685402635</v>
-      </c>
-      <c r="L15" t="n">
-        <v>-0.3226544622425629</v>
-      </c>
-      <c r="M15" t="n">
-        <v>0.008162173427013177</v>
-      </c>
-      <c r="N15" t="b">
-        <v>1</v>
-      </c>
-      <c r="O15" t="n">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>gemini</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>NearestNeighbor</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>tau</t>
-        </is>
-      </c>
-      <c r="D16" t="n">
-        <v>5</v>
-      </c>
-      <c r="E16" t="n">
-        <v>195</v>
-      </c>
-      <c r="F16" t="n">
-        <v>132</v>
-      </c>
-      <c r="G16" t="n">
-        <v>0.2984615384615385</v>
-      </c>
-      <c r="H16" t="n">
-        <v>0.3743589743589744</v>
-      </c>
-      <c r="I16" t="n">
-        <v>-0.0758974358974359</v>
-      </c>
-      <c r="J16" t="n">
-        <v>3845.5</v>
-      </c>
-      <c r="K16" t="n">
-        <v>0.2158723041617826</v>
-      </c>
-      <c r="L16" t="n">
-        <v>-0.1238323080428344</v>
-      </c>
-      <c r="M16" t="n">
-        <v>0.2158723041617826</v>
-      </c>
-      <c r="N16" t="b">
-        <v>0</v>
-      </c>
-      <c r="O16" t="n">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>gemini</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>NearestNeighbor</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>Top-1</t>
-        </is>
-      </c>
-      <c r="D17" t="n">
-        <v>5</v>
-      </c>
-      <c r="E17" t="n">
-        <v>195</v>
-      </c>
-      <c r="F17" t="n">
-        <v>96</v>
-      </c>
-      <c r="G17" t="n">
-        <v>0.4748717948717948</v>
-      </c>
-      <c r="H17" t="n">
-        <v>0.6461538461538462</v>
-      </c>
-      <c r="I17" t="n">
-        <v>-0.1712820512820513</v>
-      </c>
-      <c r="J17" t="n">
-        <v>1367.5</v>
-      </c>
-      <c r="K17" t="n">
-        <v>0.0002519173754712348</v>
-      </c>
-      <c r="L17" t="n">
-        <v>-0.4125859106529209</v>
-      </c>
-      <c r="M17" t="n">
-        <v>0.001511504252827409</v>
-      </c>
-      <c r="N17" t="b">
-        <v>1</v>
-      </c>
-      <c r="O17" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>